<commit_message>
Collated 2024 H2S data
Checked against metadata and fixed sample IDs
</commit_message>
<xml_diff>
--- a/processing_scripts/Sulfide/2024/Raw Data/TEMPEST20240624_H2S.xlsx
+++ b/processing_scripts/Sulfide/2024/Raw Data/TEMPEST20240624_H2S.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20346"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\microplate\Desktop\BioGeoChem_Microplates\COMPASS\TEMPEST\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sinet-my.sharepoint.com/personal/readz_si_edu1/Documents/TEMPEST_Porewater/processing_scripts/Sulfide/2024/Raw Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81C665E9-AB89-45F8-8E13-2225F1AB4B0D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{81C665E9-AB89-45F8-8E13-2225F1AB4B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E147060-17B8-4DA1-B743-B0BBCCF5512B}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14370" windowHeight="7350" activeTab="3" xr2:uid="{217D31C7-3677-45E3-B772-062F6D24D7E9}"/>
+    <workbookView xWindow="-19320" yWindow="690" windowWidth="19440" windowHeight="14880" activeTab="1" xr2:uid="{217D31C7-3677-45E3-B772-062F6D24D7E9}"/>
   </bookViews>
   <sheets>
     <sheet name="Lab Check" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,17 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -812,6 +823,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -819,7 +831,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1185,6 +1196,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1192,7 +1204,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1558,6 +1569,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1565,7 +1577,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3384,9 +3395,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3424,7 +3435,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3530,7 +3541,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3672,7 +3683,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4115,7 +4126,7 @@
   <dimension ref="A2:N22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="11.42578125" customWidth="1"/>
+    <col min="5" max="13" width="39.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -4890,6 +4901,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{292D26F3-DC46-4856-B879-BEE519F34DB3}">
   <dimension ref="A3:N23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="13" width="33.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -5662,6 +5676,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B531F4E6-2BC7-4F8D-97B2-8C40592F78E1}">
   <dimension ref="A3:N23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="14" width="32" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>

</xml_diff>